<commit_message>
Update blank template v3: fix theme validation error, move Nick Name to Property Info
</commit_message>
<xml_diff>
--- a/templates/AGX_Blank_Template.xlsx
+++ b/templates/AGX_Blank_Template.xlsx
@@ -14,326 +14,6 @@
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-  </numFmts>
-  <fonts count="11">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001B3A5C"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00444444"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001B3A5C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001B3A5C"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-  </fonts>
-  <fills count="7">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B8541"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F8F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5E8D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="6">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="32">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -375,7 +55,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n"/>
+      <c r="A3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="4" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -415,7 +95,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Nick Name</t>
+          <t>Project Type</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -428,7 +108,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Project Type</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B9" s="7" t="n"/>
@@ -441,7 +121,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Created Date</t>
         </is>
       </c>
       <c r="B10" s="7" t="n"/>
@@ -454,7 +134,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Created Date</t>
+          <t>Salesperson</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
@@ -467,7 +147,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Salesperson</t>
+          <t>Market</t>
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
@@ -480,45 +160,45 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Market</t>
+          <t>Estimate ID</t>
         </is>
       </c>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
-      <c r="D13" s="8" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Estimate ID</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Property Information</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Property Information</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Nick Name</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="8" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -528,7 +208,7 @@
       </c>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
-      <c r="D17" s="8" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
@@ -541,7 +221,7 @@
       </c>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
-      <c r="D18" s="9" t="inlineStr"/>
+      <c r="D18" s="8" t="inlineStr"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="n"/>
@@ -554,7 +234,7 @@
       </c>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
-      <c r="D19" s="8" t="inlineStr"/>
+      <c r="D19" s="9" t="inlineStr"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="n"/>
@@ -567,7 +247,7 @@
       </c>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
-      <c r="D20" s="9" t="inlineStr"/>
+      <c r="D20" s="8" t="inlineStr"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="n"/>
@@ -580,7 +260,7 @@
       </c>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
-      <c r="D21" s="8" t="inlineStr"/>
+      <c r="D21" s="9" t="inlineStr"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="n"/>
@@ -593,7 +273,7 @@
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
-      <c r="D22" s="9" t="inlineStr"/>
+      <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="7" t="n"/>
       <c r="G22" s="7" t="n"/>
@@ -606,7 +286,7 @@
       </c>
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="n"/>
-      <c r="D23" s="8" t="inlineStr"/>
+      <c r="D23" s="9" t="inlineStr"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="7" t="n"/>
@@ -619,7 +299,7 @@
       </c>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
-      <c r="D24" s="9" t="inlineStr"/>
+      <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="7" t="n"/>
       <c r="G24" s="7" t="n"/>
@@ -901,19 +581,18 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D14:G14"/>
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="D23:G23"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
     <mergeCell ref="D20:G20"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="D19:G19"/>
     <mergeCell ref="D10:G10"/>
     <mergeCell ref="A20:C20"/>
@@ -925,7 +604,6 @@
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="D21:G21"/>
-    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D13:G13"/>
@@ -934,11 +612,13 @@
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A3:G3"/>
+    <mergeCell ref="D16:G16"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>

</xml_diff>